<commit_message>
latest boprc biovol data
</commit_message>
<xml_diff>
--- a/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20260219 (1).xlsx
+++ b/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20260219 (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://boprc-my.sharepoint.com/personal/amber_sutherland_boprc_govt_nz/Documents/Desktop/Amber Sutherland 2025-2026/Cyanobacteria weekly results 2025-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://waikatouniversitynz-my.sharepoint.com/personal/whitney_woelmer_waikato_ac_nz/Documents/Desktop/lakecast_rotorua/data/boprc_cyano/og_excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{806F90AC-9822-47C4-9B4A-F393115C7021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{806F90AC-9822-47C4-9B4A-F393115C7021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4931F6C-B7F5-4D1A-B643-C36A03004F56}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="86280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lakes Data" sheetId="2" r:id="rId1"/>
@@ -541,16 +541,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -569,7 +570,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46072.465846990737" refreshedVersion="8" recordCount="74" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46128.427085995369" refreshedVersion="8" recordCount="74" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P75" sheet="Lakes Data"/>
   </cacheSource>
@@ -654,7 +655,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46072.465847916668" refreshedVersion="8" recordCount="13" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46128.427086111114" refreshedVersion="8" recordCount="13" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P14" sheet="Toxin Data"/>
   </cacheSource>
@@ -741,7 +742,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46072.465848148146" refreshedVersion="8" recordCount="74" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46128.427086342592" refreshedVersion="8" recordCount="74" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P75" sheet="Lakes Data"/>
   </cacheSource>
@@ -3739,7 +3740,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="AlertWarning" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="AlertWarning" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A8:D23" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="16">
     <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
@@ -3864,125 +3865,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="AlertWarning" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
-  <location ref="A37:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
-  <pivotFields count="16">
-    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-      </items>
-    </pivotField>
-    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="13">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-      </items>
-    </pivotField>
-    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="1">
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="CellsPerMl" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="TotalBioVolume" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="ToxinCluster" compact="0" outline="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="1"/>
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="13">
-    <i>
-      <x/>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="6"/>
-    </i>
-    <i r="1">
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="5"/>
-    </i>
-    <i r="1">
-      <x v="8"/>
-    </i>
-    <i r="1">
-      <x v="9"/>
-    </i>
-    <i r="1">
-      <x v="12"/>
-    </i>
-    <i>
-      <x v="3"/>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="4"/>
-      <x v="11"/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="3"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="TotalBioVolume" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="CellsPermL" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A8:D22" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="16">
@@ -4094,6 +3976,125 @@
   </colItems>
   <dataFields count="1">
     <dataField name="CellsPerMl" fld="11" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="AlertWarning" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+  <location ref="A37:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
+  <pivotFields count="16">
+    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+      </items>
+    </pivotField>
+    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="13">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+      </items>
+    </pivotField>
+    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="CellsPerMl" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="TotalBioVolume" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="ToxinCluster" compact="0" outline="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="13">
+    <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="6"/>
+    </i>
+    <i r="1">
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="5"/>
+    </i>
+    <i r="1">
+      <x v="8"/>
+    </i>
+    <i r="1">
+      <x v="9"/>
+    </i>
+    <i r="1">
+      <x v="12"/>
+    </i>
+    <i>
+      <x v="3"/>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="4"/>
+      <x v="11"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="3"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="TotalBioVolume" fld="12" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
   <extLst>
@@ -4440,27 +4441,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P75"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="28.54296875" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" customWidth="1"/>
-    <col min="9" max="9" width="20.7265625" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" customWidth="1"/>
-    <col min="12" max="12" width="18.26953125" customWidth="1"/>
-    <col min="13" max="13" width="21.453125" customWidth="1"/>
-    <col min="14" max="14" width="23.453125" customWidth="1"/>
-    <col min="15" max="15" width="27.36328125" customWidth="1"/>
-    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="12.47265625" customWidth="1"/>
+    <col min="2" max="2" width="11.7890625" customWidth="1"/>
+    <col min="3" max="3" width="13.7890625" customWidth="1"/>
+    <col min="4" max="4" width="14.7890625" customWidth="1"/>
+    <col min="5" max="5" width="18.62890625" customWidth="1"/>
+    <col min="6" max="6" width="14.47265625" customWidth="1"/>
+    <col min="7" max="7" width="28.5234375" customWidth="1"/>
+    <col min="8" max="8" width="16.62890625" customWidth="1"/>
+    <col min="9" max="9" width="20.734375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.7890625" customWidth="1"/>
+    <col min="12" max="12" width="18.26171875" customWidth="1"/>
+    <col min="13" max="13" width="21.47265625" customWidth="1"/>
+    <col min="14" max="14" width="23.47265625" customWidth="1"/>
+    <col min="15" max="15" width="27.3671875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4510,7 +4511,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -4557,7 +4558,7 @@
         <v>0.14669321939999999</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -4607,7 +4608,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -4654,7 +4655,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -4698,7 +4699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -4745,7 +4746,7 @@
         <v>6.4111904999999997E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -4795,7 +4796,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -4839,7 +4840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -4883,7 +4884,7 @@
         <v>1.014E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -4927,7 +4928,7 @@
         <v>1.40634E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -4971,7 +4972,7 @@
         <v>2.6600000000000001E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -5015,7 +5016,7 @@
         <v>5.7000000000000002E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>43</v>
       </c>
@@ -5062,7 +5063,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -5106,7 +5107,7 @@
         <v>0.18661050000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -5153,7 +5154,7 @@
         <v>7.9782364999999994E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -5197,7 +5198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>50</v>
       </c>
@@ -5241,7 +5242,7 @@
         <v>1.554E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>52</v>
       </c>
@@ -5285,7 +5286,7 @@
         <v>1.248E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -5329,7 +5330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -5373,7 +5374,7 @@
         <v>8.5722000000000003E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -5420,7 +5421,7 @@
         <v>0.43043337701388901</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -5464,7 +5465,7 @@
         <v>3.04420770833333E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -5508,7 +5509,7 @@
         <v>1.9603566666666701E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -5552,7 +5553,7 @@
         <v>7.6266899999999999E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>64</v>
       </c>
@@ -5599,7 +5600,7 @@
         <v>1.484945E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>65</v>
       </c>
@@ -5646,7 +5647,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
         <v>66</v>
       </c>
@@ -5690,7 +5691,7 @@
         <v>1.4300000000000001E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -5734,7 +5735,7 @@
         <v>4.9529999999999995E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
         <v>69</v>
       </c>
@@ -5778,7 +5779,7 @@
         <v>7.8100000000000001E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
         <v>71</v>
       </c>
@@ -5822,7 +5823,7 @@
         <v>0.25746839999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -5866,7 +5867,7 @@
         <v>2.129868E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
         <v>73</v>
       </c>
@@ -5913,7 +5914,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -5960,7 +5961,7 @@
         <v>1.924E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
         <v>75</v>
       </c>
@@ -6004,7 +6005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>76</v>
       </c>
@@ -6048,7 +6049,7 @@
         <v>1.17E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -6095,7 +6096,7 @@
         <v>6.7522572000000003E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -6145,7 +6146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -6189,7 +6190,7 @@
         <v>8.8800000000000001E-4</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -6233,7 +6234,7 @@
         <v>1.0920000000000001E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>83</v>
       </c>
@@ -6277,7 +6278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -6321,7 +6322,7 @@
         <v>0.21068054999999999</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>85</v>
       </c>
@@ -6368,7 +6369,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>88</v>
       </c>
@@ -6412,7 +6413,7 @@
         <v>0.23069385000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>89</v>
       </c>
@@ -6456,7 +6457,7 @@
         <v>3.2869044E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>90</v>
       </c>
@@ -6500,7 +6501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -6544,7 +6545,7 @@
         <v>1.0619E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" t="s">
         <v>92</v>
       </c>
@@ -6588,7 +6589,7 @@
         <v>8.7399999999999999E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
         <v>93</v>
       </c>
@@ -6632,7 +6633,7 @@
         <v>1.248E-4</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
         <v>94</v>
       </c>
@@ -6679,7 +6680,7 @@
         <v>2.37244E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -6723,7 +6724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -6770,7 +6771,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -6814,7 +6815,7 @@
         <v>1.786E-3</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" t="s">
         <v>99</v>
       </c>
@@ -6858,7 +6859,7 @@
         <v>0.1076391</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" t="s">
         <v>100</v>
       </c>
@@ -6905,7 +6906,7 @@
         <v>3.4084400000000001E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" t="s">
         <v>102</v>
       </c>
@@ -6949,7 +6950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" t="s">
         <v>103</v>
       </c>
@@ -6993,7 +6994,7 @@
         <v>3.542E-3</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" t="s">
         <v>104</v>
       </c>
@@ -7037,7 +7038,7 @@
         <v>7.4100000000000001E-4</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" t="s">
         <v>105</v>
       </c>
@@ -7084,7 +7085,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" t="s">
         <v>106</v>
       </c>
@@ -7131,7 +7132,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A60" t="s">
         <v>108</v>
       </c>
@@ -7175,7 +7176,7 @@
         <v>1.48E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A61" t="s">
         <v>109</v>
       </c>
@@ -7219,7 +7220,7 @@
         <v>7.0200000000000004E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A62" t="s">
         <v>110</v>
       </c>
@@ -7263,7 +7264,7 @@
         <v>4.0870439999999997E-3</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A63" t="s">
         <v>111</v>
       </c>
@@ -7307,7 +7308,7 @@
         <v>9.0330300000000002E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" t="s">
         <v>112</v>
       </c>
@@ -7351,7 +7352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A65" t="s">
         <v>116</v>
       </c>
@@ -7398,7 +7399,7 @@
         <v>4.5049586400000001E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A66" t="s">
         <v>117</v>
       </c>
@@ -7442,7 +7443,7 @@
         <v>6.9930000000000001E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -7489,7 +7490,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A68" t="s">
         <v>119</v>
       </c>
@@ -7533,7 +7534,7 @@
         <v>4.6799999999999999E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A69" t="s">
         <v>120</v>
       </c>
@@ -7577,7 +7578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A70" t="s">
         <v>121</v>
       </c>
@@ -7621,7 +7622,7 @@
         <v>0.1871514</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A71" t="s">
         <v>122</v>
       </c>
@@ -7668,7 +7669,7 @@
         <v>2.37133E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A72" t="s">
         <v>124</v>
       </c>
@@ -7712,7 +7713,7 @@
         <v>6.4471679999999996E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A73" t="s">
         <v>125</v>
       </c>
@@ -7756,7 +7757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A74" t="s">
         <v>126</v>
       </c>
@@ -7800,7 +7801,7 @@
         <v>2.1635999999999999E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A75" t="s">
         <v>127</v>
       </c>
@@ -7858,27 +7859,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="22.26953125" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" customWidth="1"/>
-    <col min="9" max="9" width="20.7265625" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" customWidth="1"/>
-    <col min="12" max="12" width="13.6328125" customWidth="1"/>
-    <col min="13" max="13" width="19.36328125" customWidth="1"/>
-    <col min="14" max="14" width="23.453125" customWidth="1"/>
-    <col min="15" max="15" width="27.36328125" customWidth="1"/>
-    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="12.47265625" customWidth="1"/>
+    <col min="2" max="2" width="11.7890625" customWidth="1"/>
+    <col min="3" max="3" width="13.7890625" customWidth="1"/>
+    <col min="4" max="4" width="14.7890625" customWidth="1"/>
+    <col min="5" max="5" width="18.62890625" customWidth="1"/>
+    <col min="6" max="6" width="14.47265625" customWidth="1"/>
+    <col min="7" max="7" width="22.26171875" customWidth="1"/>
+    <col min="8" max="8" width="16.62890625" customWidth="1"/>
+    <col min="9" max="9" width="20.734375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.7890625" customWidth="1"/>
+    <col min="12" max="12" width="13.62890625" customWidth="1"/>
+    <col min="13" max="13" width="19.3671875" customWidth="1"/>
+    <col min="14" max="14" width="23.47265625" customWidth="1"/>
+    <col min="15" max="15" width="27.3671875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7928,7 +7929,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -7978,7 +7979,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -8025,7 +8026,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -8075,7 +8076,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>43</v>
       </c>
@@ -8122,7 +8123,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -8169,7 +8170,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -8216,7 +8217,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>79</v>
       </c>
@@ -8266,7 +8267,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>85</v>
       </c>
@@ -8313,7 +8314,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>97</v>
       </c>
@@ -8360,7 +8361,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>105</v>
       </c>
@@ -8407,7 +8408,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>106</v>
       </c>
@@ -8454,7 +8455,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>118</v>
       </c>
@@ -8501,7 +8502,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>127</v>
       </c>
@@ -8559,15 +8560,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="32.08984375" customWidth="1"/>
-    <col min="3" max="3" width="17.08984375" customWidth="1"/>
-    <col min="4" max="4" width="23.1796875" customWidth="1"/>
+    <col min="2" max="2" width="32.1015625" customWidth="1"/>
+    <col min="3" max="3" width="17.1015625" customWidth="1"/>
+    <col min="4" max="4" width="23.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>128</v>
       </c>
@@ -8575,7 +8576,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>130</v>
       </c>
@@ -8583,7 +8584,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>131</v>
       </c>
@@ -8591,7 +8592,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>133</v>
       </c>
@@ -8599,7 +8600,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C8" s="6" t="s">
         <v>148</v>
       </c>
@@ -8607,12 +8608,12 @@
         <v>149</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -8626,161 +8627,161 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>0.21648618105708797</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="7">
         <v>0.21629200605708798</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" t="s">
         <v>31</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>0.10434984410000001</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="7">
         <v>0.10428864410000001</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>78</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>0.33386931269999998</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="7">
         <v>0.3338162127</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" t="s">
         <v>107</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>9.7817455999999997E-2</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="7">
         <v>9.7817455999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>41</v>
       </c>
       <c r="B15" t="s">
         <v>42</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>0.28385831499999997</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="7">
         <v>0.28383156499999995</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B16" t="s">
         <v>63</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>9.4050850000000005E-2</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="7">
         <v>9.4050850000000005E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>57</v>
       </c>
       <c r="B17" t="s">
         <v>58</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>0.46283581076388897</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="7">
         <v>0.46283581076388897</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" t="s">
         <v>70</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>0.31286575899999991</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="7">
         <v>0.31247560899999993</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" t="s">
         <v>95</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>0.13389067199999999</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="7">
         <v>0.133796622</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" t="s">
         <v>101</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>4.0073906000000006E-2</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="7">
         <v>3.9928106000000005E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" t="s">
         <v>123</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>5.2292818999999997E-2</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="7">
         <v>5.2215193999999999E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>86</v>
       </c>
       <c r="B22" t="s">
         <v>87</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>0.28839704099999997</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="7">
         <v>0.28819926599999995</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>113</v>
       </c>
       <c r="B23" t="s">
         <v>114</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="7">
         <v>0.2414859114</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="7">
         <v>0.24148028639999999</v>
       </c>
     </row>
@@ -8792,15 +8793,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" customWidth="1"/>
-    <col min="2" max="2" width="33.7265625" customWidth="1"/>
-    <col min="3" max="3" width="31.36328125" customWidth="1"/>
-    <col min="4" max="4" width="29.54296875" customWidth="1"/>
+    <col min="1" max="1" width="24.62890625" customWidth="1"/>
+    <col min="2" max="2" width="33.734375" customWidth="1"/>
+    <col min="3" max="3" width="31.3671875" customWidth="1"/>
+    <col min="4" max="4" width="29.5234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>135</v>
       </c>
@@ -8814,7 +8815,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>139</v>
       </c>
@@ -8828,7 +8829,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>140</v>
       </c>
@@ -8842,7 +8843,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>144</v>
       </c>
@@ -8856,7 +8857,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
@@ -8867,12 +8868,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -8883,138 +8884,138 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="7">
         <v>369.65999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" t="s">
         <v>31</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="7">
         <v>135.27000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>78</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="7">
         <v>281.79000000000002</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" t="s">
         <v>107</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="7">
         <v>6.4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>41</v>
       </c>
       <c r="B15" t="s">
         <v>42</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="7">
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B16" t="s">
         <v>63</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="7">
         <v>11.6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>57</v>
       </c>
       <c r="B17" t="s">
         <v>70</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="7">
         <v>71.3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" t="s">
         <v>95</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="7">
         <v>3.4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" t="s">
         <v>101</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="7">
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B20" t="s">
         <v>123</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="7">
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>86</v>
       </c>
       <c r="B21" t="s">
         <v>87</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="7">
         <v>68.400000000000006</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>113</v>
       </c>
       <c r="B22" t="s">
         <v>114</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="7">
         <v>20.9</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="3" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="4" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="5" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="6" t="s">
         <v>12</v>
       </c>
@@ -9022,7 +9023,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="6" t="s">
         <v>1</v>
       </c>
@@ -9033,122 +9034,122 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>17</v>
       </c>
       <c r="B39" t="s">
         <v>18</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="7">
         <v>0.21648618105708797</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B40" t="s">
         <v>31</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="7">
         <v>0.10434984410000001</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B41" t="s">
         <v>78</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="7">
         <v>0.33386931269999998</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B42" t="s">
         <v>107</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="7">
         <v>9.7817455999999997E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>41</v>
       </c>
       <c r="B43" t="s">
         <v>42</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="7">
         <v>0.28385831499999997</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B44" t="s">
         <v>63</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="7">
         <v>9.4050850000000005E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>57</v>
       </c>
       <c r="B45" t="s">
         <v>58</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="7">
         <v>0.46283581076388897</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B46" t="s">
         <v>70</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="7">
         <v>0.31286575899999991</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B47" t="s">
         <v>95</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="7">
         <v>0.13389067199999999</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B48" t="s">
         <v>101</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="7">
         <v>4.0073906000000006E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B49" t="s">
         <v>123</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="7">
         <v>5.2292818999999997E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>86</v>
       </c>
       <c r="B50" t="s">
         <v>87</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="7">
         <v>0.28839704099999997</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>113</v>
       </c>
       <c r="B51" t="s">
         <v>114</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="7">
         <v>0.2414859114</v>
       </c>
     </row>

</xml_diff>